<commit_message>
feat: packing machine catalog + selector, grinding menu hub and spec fixes
- Add "Máy nghiền & đóng gói" hub between Home and the grinding module
- Add packing machine catalog (7 series, 20 models) from the supplier
  catalog as a read-only JSON asset, with cleaned machine images
  (watermark and background removed), series/detail/search/compare
  screens, share text/PDF, and a "Chọn máy phù hợp" selector using the
  same MATCH / NOT_MATCH / UNKNOWN logic as the grinding selector
- Share catalog PDF builder and feature list widget between modules
- SpecRow: choose layout from measured text width instead of char count
- Grinding: sort models numerically, split multi-clause input size into
  lines, drop "Ghi chú" from application details, remove supplier
  mention from ASG structure (seed databaseVersion 2.2.19)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/grinding_machine/ai_ready.xlsx
+++ b/test/fixtures/grinding_machine/ai_ready.xlsx
@@ -2534,7 +2534,7 @@
     <t xml:space="preserve">STRONG CANDIDATE</t>
   </si>
   <si>
-    <t xml:space="preserve">2.2.18</t>
+    <t xml:space="preserve">2.2.19</t>
   </si>
   <si>
     <t xml:space="preserve">Roller mill</t>
@@ -2604,8 +2604,7 @@
 Máy sử dụng chuyển động tương đối giữa bộ phận cố định và búa/dao chuyển động để nghiền nguyên liệu bằng tác động va đập kết hợp lực ly tâm. Nhà sản xuất cho biết máy phù hợp với các nguyên liệu như tiêu, gia vị, hạt thì là...</t>
   </si>
   <si>
-    <t xml:space="preserve">Theo Brightsail, bộ BSG self-priming grinding unit gồm:
-- Máy nghiền chính
+    <t xml:space="preserve">- Máy nghiền chính
 - Thiết bị phụ trợ
 - Đường ống vận chuyển
 - Tủ/thiết bị điều khiển điện

</xml_diff>